<commit_message>
Improve repo formatting and README.md to match research paper
</commit_message>
<xml_diff>
--- a/SSC7/Grading/2 stage/6-examples/SSC7_Grading_2-stage_2026-03-12_6-examples_Gemini3.1ProPreviewGeneration_GPT5.5AutoGrading.xlsx
+++ b/SSC7/Grading/2 stage/6-examples/SSC7_Grading_2-stage_2026-03-12_6-examples_Gemini3.1ProPreviewGeneration_GPT5.5AutoGrading.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marc-antoinenadeau/Desktop/B.Eng Software Engineering /7th Semester/Capstone/Code/Evaluations/SSC7/Grading/2 stage/6-examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D834E7C8-0074-9344-9031-4A2933644B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{56E364A6-4D49-854D-A438-5DC64E3F2760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17640" yWindow="-21000" windowWidth="30240" windowHeight="17300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17640" yWindow="-21000" windowWidth="30240" windowHeight="17300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SSC7" sheetId="1" r:id="rId1"/>
@@ -13225,6 +13225,10 @@
       </c>
       <c r="D7" s="45">
         <f>SUMIF('GPT-5.5 Grading'!$A$68:$A$74, $A7, 'GPT-5.5 Grading'!$C$68:$C$74)</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="45">
+        <f>COUNTIFS('GPT-5.5 Grading'!$A$2:$A$67, $A7, 'GPT-5.5 Grading'!$C$2:$C$67,0)</f>
         <v>0</v>
       </c>
       <c r="F7" s="45" t="str">

</xml_diff>